<commit_message>
modelo LightGBM segunda versión mejorada.
</commit_message>
<xml_diff>
--- a/07_seleccion_entrenar_modelo/3_entrenar_modelo_arimax/2_con_rezago_sin_escalado_sin_reduccion_aicc/2_datos/1_raw/df_meteo_epi_sin_rezagos.xlsx
+++ b/07_seleccion_entrenar_modelo/3_entrenar_modelo_arimax/2_con_rezago_sin_escalado_sin_reduccion_aicc/2_datos/1_raw/df_meteo_epi_sin_rezagos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\investigacion\arima\2_ejecucion_plan_trabajo\07_seleccion_entrenar_modelo\2_entrenar_modelo\2_entrenar_modelo_con_rezago_sin_escalado_sin_reduccion\2_datos\1_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\investigacion\arima\07_seleccion_entrenar_modelo\3_entrenar_modelo_arimax\2_con_rezago_sin_escalado_sin_reduccion_aicc\2_datos\1_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FAD454-3D20-4F6C-8549-53BEA08A17D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5D2D8A-C2F3-4FF0-993D-711AFECC24FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -440,6 +440,7 @@
     <col min="5" max="5" width="15.33203125" customWidth="1"/>
     <col min="6" max="6" width="18.21875" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>